<commit_message>
Fix dodge input facing and unify per-frame player input sampling.
Dodge was applying empty tag-track effects as full skill damage on self, and later reused locomotion move intent as facing, so rolls could self-hit, keep the old stick direction, or keep walking after release. Sample WASD/joystick once into PlayerInputSnapshot after EventSystem, keep LastAim for dodge only, and submit slot skills in CombatEntity.Update before ActSpell so enqueue and cast share the same frame.

Also land ZZZ/WuWa-style gait (Ctrl walk/jog, Shift sprint latch), camera-relative roll start, joystick tap aiming, damage-text/passive-buff wiring, and drop unused locomotion test scenes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Config/Datas/AbilitySetting.xlsx
+++ b/Tools/Config/Datas/AbilitySetting.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ACTGameEditor\Tools\Config\Datas\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6880"/>
+    <workbookView windowWidth="18350" windowHeight="6880" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="主动技能" sheetId="1" r:id="rId1"/>
     <sheet name="被动技能" sheetId="2" r:id="rId2"/>
-    <sheet name="主动技能伤害倍率" sheetId="4" r:id="rId3"/>
+    <sheet name="主动技能伤害倍率" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,20 +43,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 从10000开始
 </t>
         </r>
@@ -61,20 +57,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 ActiveSkill是主动
 PassiveSkill是被动
 </t>
@@ -85,20 +72,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 1为自身
 2为己方
 3为敌方</t>
@@ -109,20 +87,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 1为手动指定
 2为碰撞检测
 3为条件指定</t>
@@ -133,20 +102,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -157,20 +117,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -181,20 +132,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -205,20 +147,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -229,20 +162,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -253,20 +177,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -277,20 +192,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -301,20 +207,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -335,20 +232,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 从10000开始
 </t>
         </r>
@@ -358,20 +246,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 ActiveSkill是主动
 PassiveSkill是被动
 </t>
@@ -382,20 +261,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 1为自身
 2为己方
 3为敌方</t>
@@ -406,20 +276,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 1为手动指定
 2为碰撞检测
 3为条件指定</t>
@@ -430,20 +291,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -464,20 +316,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 从10000开始
 </t>
         </r>
@@ -487,20 +330,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t xml:space="preserve">admin:
 ActiveSkill是主动
 PassiveSkill是被动
 </t>
@@ -511,20 +345,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 1为自身
 2为己方
 3为敌方</t>
@@ -535,20 +360,11 @@
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
+            <sz val="10"/>
             <rFont val="宋体"/>
             <charset val="134"/>
           </rPr>
-          <t>admin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="宋体"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>admin:
 #号分割
 第一个是方法名
 后面的均为参数</t>
@@ -560,7 +376,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="68">
   <si>
     <t>##var</t>
   </si>
@@ -695,6 +511,24 @@
   </si>
   <si>
     <t>普攻3</t>
+  </si>
+  <si>
+    <t>时空断裂闪避</t>
+  </si>
+  <si>
+    <t>攻击后加攻</t>
+  </si>
+  <si>
+    <t>PassiveSkill</t>
+  </si>
+  <si>
+    <t>释放普攻或大招后 5 秒内攻击力提升 20%，重复攻击刷新时间</t>
+  </si>
+  <si>
+    <t>命中点燃</t>
+  </si>
+  <si>
+    <t>主动技能攻击命中后给敌人施加点燃</t>
   </si>
   <si>
     <t>SkillName</t>
@@ -759,7 +593,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -969,13 +803,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
+      <sz val="10"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
@@ -1458,48 +1286,48 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="22" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="23" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="22" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="23" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="22" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="23" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="22" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="23" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1811,366 +1639,372 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="3" max="3" width="16.8181818181818" customWidth="1"/>
-    <col min="4" max="4" width="17.4545454545455" customWidth="1"/>
-    <col min="5" max="5" width="20.8181818181818" customWidth="1"/>
-    <col min="6" max="6" width="20.3636363636364" customWidth="1"/>
-    <col min="7" max="7" width="17.3636363636364" customWidth="1"/>
-    <col min="8" max="8" width="19.4545454545455" customWidth="1"/>
-    <col min="9" max="9" width="28.4545454545455" customWidth="1"/>
-    <col min="10" max="10" width="22.8181818181818" customWidth="1"/>
-    <col min="11" max="12" width="24.2727272727273" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
-    <col min="14" max="14" width="23" customWidth="1"/>
-    <col min="15" max="15" width="21.4545454545455" customWidth="1"/>
-    <col min="16" max="16" width="19.4545454545455" customWidth="1"/>
-    <col min="17" max="17" width="22.4545454545455" customWidth="1"/>
+    <col min="3" max="3" width="16.8181818181818" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.4545454545455" style="2" customWidth="1"/>
+    <col min="5" max="5" width="20.8181818181818" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.3636363636364" style="2" customWidth="1"/>
+    <col min="7" max="7" width="17.3636363636364" style="2" customWidth="1"/>
+    <col min="8" max="8" width="19.4545454545455" style="2" customWidth="1"/>
+    <col min="9" max="9" width="28.4545454545455" style="2" customWidth="1"/>
+    <col min="10" max="10" width="22.8181818181818" style="2" customWidth="1"/>
+    <col min="11" max="12" width="24.2727272727273" style="2" customWidth="1"/>
+    <col min="13" max="13" width="22" style="2" customWidth="1"/>
+    <col min="14" max="14" width="23" style="2" customWidth="1"/>
+    <col min="15" max="15" width="21.4545454545455" style="2" customWidth="1"/>
+    <col min="16" max="16" width="19.4545454545455" style="2" customWidth="1"/>
+    <col min="17" max="17" width="22.4545454545455" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="17" customFormat="1" spans="1:31">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="18" customFormat="1" spans="1:31">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="20"/>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="20"/>
-      <c r="Z1" s="20"/>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="20"/>
-      <c r="AE1" s="20"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="21"/>
+      <c r="AA1" s="21"/>
+      <c r="AB1" s="21"/>
+      <c r="AC1" s="21"/>
+      <c r="AD1" s="21"/>
+      <c r="AE1" s="21"/>
     </row>
-    <row r="2" s="18" customFormat="1" spans="1:31">
-      <c r="A2" s="2" t="s">
+    <row r="2" s="19" customFormat="1" spans="1:31">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
-      <c r="Z2" s="21"/>
-      <c r="AA2" s="21"/>
-      <c r="AB2" s="21"/>
-      <c r="AC2" s="21"/>
-      <c r="AD2" s="21"/>
-      <c r="AE2" s="21"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
     </row>
-    <row r="3" s="19" customFormat="1" spans="1:31">
-      <c r="A3" s="7" t="s">
+    <row r="3" s="20" customFormat="1" spans="1:31">
+      <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="O3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="P3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Q3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20"/>
-      <c r="T3" s="20"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="20"/>
-      <c r="Y3" s="20"/>
-      <c r="Z3" s="20"/>
-      <c r="AA3" s="20"/>
-      <c r="AB3" s="20"/>
-      <c r="AC3" s="20"/>
-      <c r="AD3" s="20"/>
-      <c r="AE3" s="20"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="21"/>
+      <c r="Y3" s="21"/>
+      <c r="Z3" s="21"/>
+      <c r="AA3" s="21"/>
+      <c r="AB3" s="21"/>
+      <c r="AC3" s="21"/>
+      <c r="AD3" s="21"/>
+      <c r="AE3" s="21"/>
     </row>
-    <row r="4" s="17" customFormat="1" spans="1:31">
-      <c r="A4" s="2" t="s">
+    <row r="4" s="18" customFormat="1" spans="1:31">
+      <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="O4" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="P4" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="Q4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
-      <c r="X4" s="20"/>
-      <c r="Y4" s="20"/>
-      <c r="Z4" s="20"/>
-      <c r="AA4" s="20"/>
-      <c r="AB4" s="20"/>
-      <c r="AC4" s="20"/>
-      <c r="AD4" s="20"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="21"/>
+      <c r="AB4" s="21"/>
+      <c r="AC4" s="21"/>
+      <c r="AD4" s="21"/>
     </row>
     <row r="5" spans="1:31">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="12" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="13" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:31">
-      <c r="A6" s="12"/>
-      <c r="B6" s="9">
+      <c r="A6" s="13"/>
+      <c r="B6" s="10">
         <v>11000</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="10">
         <v>1</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="10">
         <v>1</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="10">
         <v>2</v>
       </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="13"/>
     </row>
     <row r="7" spans="1:31">
-      <c r="A7" s="12"/>
-      <c r="B7" s="9">
+      <c r="A7" s="13"/>
+      <c r="B7" s="10">
         <v>11001</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="10">
         <v>3</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="10">
         <v>2</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="10">
         <v>0</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="12"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="13"/>
     </row>
     <row r="8" spans="1:31">
-      <c r="A8" s="12"/>
-      <c r="B8" s="9">
+      <c r="A8" s="13"/>
+      <c r="B8" s="10">
         <v>11002</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="10">
         <v>3</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="10">
         <v>2</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="10">
         <v>0</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="12"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="13"/>
     </row>
     <row r="9" spans="1:31">
-      <c r="A9" s="12"/>
-      <c r="B9" s="9">
+      <c r="A9" s="13"/>
+      <c r="B9" s="10">
         <v>11003</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="10">
         <v>3</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="10">
         <v>2</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="10">
         <v>0</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="12"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" spans="1:31">
+      <c r="B10">
+        <v>11004</v>
+      </c>
+      <c r="C10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -2197,131 +2031,249 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
+  <dimension ref="A1:Q7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="6"/>
   <cols>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="13.3636363636364" customWidth="1"/>
-    <col min="5" max="5" width="17.6363636363636" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="18.3636363636364" customWidth="1"/>
-    <col min="8" max="8" width="21.6363636363636" customWidth="1"/>
-    <col min="9" max="9" width="33" customWidth="1"/>
+    <col min="3" max="3" width="14" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.3636363636364" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17.6363636363636" style="2" customWidth="1"/>
+    <col min="6" max="6" width="22" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.3636363636364" style="2" customWidth="1"/>
+    <col min="8" max="8" width="21.6363636363636" style="2" customWidth="1"/>
+    <col min="9" max="9" width="33" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:17">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:17">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:17">
+      <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>19</v>
       </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
+        <v>18</v>
+      </c>
+      <c r="O3" t="s">
+        <v>18</v>
+      </c>
+      <c r="P3" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:17">
+      <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K4" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" t="s">
+        <v>34</v>
+      </c>
+      <c r="M4" t="s">
+        <v>34</v>
+      </c>
+      <c r="N4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O4" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:17">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="12" t="s">
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="13" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="B6">
+        <v>19001</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="B7">
+        <v>19002</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2343,191 +2295,191 @@
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14" outlineLevelRow="7" outlineLevelCol="7"/>
   <cols>
-    <col min="3" max="3" width="16.4545454545455" customWidth="1"/>
-    <col min="4" max="4" width="13.2727272727273" customWidth="1"/>
-    <col min="5" max="5" width="19.7272727272727" customWidth="1"/>
-    <col min="6" max="6" width="20.3636363636364" customWidth="1"/>
-    <col min="7" max="7" width="17.6363636363636" customWidth="1"/>
-    <col min="8" max="8" width="25.2727272727273" customWidth="1"/>
-    <col min="9" max="9" width="16.8181818181818" customWidth="1"/>
-    <col min="10" max="10" width="15.3636363636364" customWidth="1"/>
-    <col min="11" max="11" width="14.2727272727273" customWidth="1"/>
-    <col min="12" max="12" width="19" customWidth="1"/>
+    <col min="3" max="3" width="16.4545454545455" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.2727272727273" style="2" customWidth="1"/>
+    <col min="5" max="5" width="19.7272727272727" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.3636363636364" style="2" customWidth="1"/>
+    <col min="7" max="7" width="17.6363636363636" style="2" customWidth="1"/>
+    <col min="8" max="8" width="25.2727272727273" style="2" customWidth="1"/>
+    <col min="9" max="9" width="16.8181818181818" style="2" customWidth="1"/>
+    <col min="10" max="10" width="15.3636363636364" style="2" customWidth="1"/>
+    <col min="11" max="11" width="14.2727272727273" style="2" customWidth="1"/>
+    <col min="12" max="12" width="19" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>50</v>
+      <c r="C1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>56</v>
+      <c r="C4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" ht="13" spans="1:8">
-      <c r="A5" s="8" t="s">
+    <row r="5" s="1" customFormat="1" ht="13" customHeight="1" spans="1:8">
+      <c r="A5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>60</v>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="12"/>
-      <c r="B6" s="9">
-        <v>11000</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9">
+      <c r="A6" s="13"/>
+      <c r="B6" s="10">
+        <v>11001</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10">
         <v>1</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="14">
         <v>1</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="14">
+      <c r="F6" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" s="15">
         <v>0</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="12"/>
-      <c r="B7" s="9">
-        <v>11001</v>
-      </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9">
+      <c r="A7" s="13"/>
+      <c r="B7" s="10">
+        <v>11002</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10">
         <v>1</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="14">
         <v>3</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G7" s="16">
+      <c r="F7" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="17">
         <v>0</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="12"/>
-      <c r="B8" s="9">
-        <v>11002</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9">
+      <c r="A8" s="13"/>
+      <c r="B8" s="10">
+        <v>11003</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10">
         <v>1</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="14">
         <v>3</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="16">
+      <c r="F8" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" s="17">
         <v>0</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="16">
         <v>1</v>
       </c>
     </row>

</xml_diff>